<commit_message>
bumping version to 0.2.0 and refreshing docs .jupyter_cache
</commit_message>
<xml_diff>
--- a/docs/howto/ame_results.xlsx
+++ b/docs/howto/ame_results.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,72 +417,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>std_error</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ci_lower</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ci_upper</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>conf_level</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>n_obs</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>term</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>statistic</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>kappa</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>fallback_triggered</t>
         </is>
@@ -546,7 +534,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.07898145839531677</v>
+        <v>0.02330207054379209</v>
       </c>
       <c r="N2" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
feat(result): GraphResult arithmetic composability and 0.4.0 docs refresh
- Add `+`, `-`, and unary `-` operators to `GraphResult` that propagate

  covariance on the inference scale for delta, simulation, and bootstrap

  results.

- Cache `Node.collect()` outputs by node hash so stochastic stages such as

  `reimpute` produce reproducible draws.

- Validate scenario/sample weights eagerly before JAX tracing to avoid

  `TracerBoolConversionError`.

- Refresh tutorials, how-to guides, demos, and API docs for the 0.4.0

  `GComputation` / `Plan` surface.

- Update regression golden files and add operator/caching tests.
</commit_message>
<xml_diff>
--- a/docs/howto/ame_results.xlsx
+++ b/docs/howto/ame_results.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,78 +413,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>std_error</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ci_lower</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ci_upper</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>conf_level</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>n_obs</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>term</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>statistic</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>kappa</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>fallback_triggered</t>
         </is>
       </c>
     </row>
@@ -546,10 +529,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.07898145839531677</v>
-      </c>
-      <c r="N2" t="b">
-        <v>0</v>
+        <v>0.02330207054379209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>